<commit_message>
feature :- chnage the emaill servive now using maildrop email services api for member register and verify
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
   <si>
     <t>Email</t>
   </si>
@@ -85,6 +85,33 @@
   </si>
   <si>
     <t>Youth Club Automation 2262</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 6287</t>
+  </si>
+  <si>
+    <t>VeolaConsidine@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 196</t>
+  </si>
+  <si>
+    <t>SammieSmitham@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 4484</t>
+  </si>
+  <si>
+    <t>BennyDickens@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 8854</t>
+  </si>
+  <si>
+    <t>CassyLubowitz@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 5874</t>
   </si>
 </sst>
 </file>
@@ -1069,7 +1096,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1168,6 +1195,46 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- issue fix and sleep time reduce
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
   <si>
     <t>Email</t>
   </si>
@@ -112,6 +112,9 @@
   </si>
   <si>
     <t>Youth Club Automation 5874</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 4770</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1099,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1235,6 +1238,14 @@
         <v>17</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- minor change in first and last name of register member
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
   <si>
     <t>Email</t>
   </si>
@@ -115,6 +115,12 @@
   </si>
   <si>
     <t>Youth Club Automation 4770</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 5183</t>
+  </si>
+  <si>
+    <t>AngeleKilbackMD@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1099,7 +1105,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1246,6 +1252,14 @@
         <v>12</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature:-no changes just run the floe and member added
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
   <si>
     <t>Email</t>
   </si>
@@ -121,6 +121,9 @@
   </si>
   <si>
     <t>AngeleKilbackMD@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 3470</t>
   </si>
 </sst>
 </file>
@@ -1105,7 +1108,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1260,6 +1263,14 @@
         <v>30</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
add yml file changes
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
   <si>
     <t>Email</t>
   </si>
@@ -127,6 +127,12 @@
   </si>
   <si>
     <t>Youth Club Automation 1473</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 6345</t>
+  </si>
+  <si>
+    <t>HassieBrown@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1111,7 +1117,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1282,6 +1288,14 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature new add data in prod excel
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
   <si>
     <t>Email</t>
   </si>
@@ -133,6 +133,9 @@
   </si>
   <si>
     <t>HassieBrown@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 4394</t>
   </si>
 </sst>
 </file>
@@ -1117,7 +1120,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1296,6 +1299,14 @@
         <v>34</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature changes in flow for more optimize
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="44">
   <si>
     <t>Email</t>
   </si>
@@ -157,6 +157,9 @@
   </si>
   <si>
     <t>Youth Club Automation 2517</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 8226</t>
   </si>
 </sst>
 </file>
@@ -1141,7 +1144,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1384,6 +1387,14 @@
         <v>34</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature time reduce and optimize code
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="46">
   <si>
     <t>Email</t>
   </si>
@@ -163,6 +163,9 @@
   </si>
   <si>
     <t>Youth Club Automation 9435</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 775</t>
   </si>
 </sst>
 </file>
@@ -1147,7 +1150,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1406,6 +1409,14 @@
         <v>34</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- Member registration thread now 3 , 2 2 set
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="49">
   <si>
     <t>Email</t>
   </si>
@@ -172,6 +172,9 @@
   </si>
   <si>
     <t>Youth Club Automation 3504</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 742</t>
   </si>
 </sst>
 </file>
@@ -1156,7 +1159,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1439,6 +1442,14 @@
         <v>34</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature test on local
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="51">
   <si>
     <t>Email</t>
   </si>
@@ -178,6 +178,9 @@
   </si>
   <si>
     <t>Youth Club Automation 6965</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 3456</t>
   </si>
 </sst>
 </file>
@@ -1162,7 +1165,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1461,6 +1464,14 @@
         <v>34</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- fixing issue due server
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="58">
   <si>
     <t>Email</t>
   </si>
@@ -199,6 +199,9 @@
   </si>
   <si>
     <t>Prerana Colony Apex Youth Club</t>
+  </si>
+  <si>
+    <t>Sahyog Vihar Nova Youth Club</t>
   </si>
 </sst>
 </file>
@@ -1183,7 +1186,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1530,6 +1533,14 @@
         <v>55</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- create youth club and approve by super admin
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="61">
   <si>
     <t>Email</t>
   </si>
@@ -208,6 +208,9 @@
   </si>
   <si>
     <t>MissWyattRau@yopmail.com</t>
+  </si>
+  <si>
+    <t>Pragati Block Alpha Youth Club</t>
   </si>
 </sst>
 </file>
@@ -1192,7 +1195,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1555,6 +1558,14 @@
         <v>59</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
after merge and run the flow modified excel file
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="62">
   <si>
     <t>Email</t>
   </si>
@@ -211,6 +211,9 @@
   </si>
   <si>
     <t>Pragati Block Alpha Youth Club</t>
+  </si>
+  <si>
+    <t>Navjyoti Ward Sigma Youth Club</t>
   </si>
 </sst>
 </file>
@@ -1195,7 +1198,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1566,6 +1569,14 @@
         <v>59</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature just run flow on local
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="64">
   <si>
     <t>Email</t>
   </si>
@@ -214,6 +214,12 @@
   </si>
   <si>
     <t>Navjyoti Ward Sigma Youth Club</t>
+  </si>
+  <si>
+    <t>Umang Sector Beta Youth Club</t>
+  </si>
+  <si>
+    <t>yco2607041223m6@maildrop.cc</t>
   </si>
 </sst>
 </file>
@@ -1198,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1577,6 +1583,14 @@
         <v>59</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :-  pull main and merge and the flow
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="68">
   <si>
     <t>Email</t>
   </si>
@@ -220,6 +220,18 @@
   </si>
   <si>
     <t>yco2607041223m6@maildrop.cc</t>
+  </si>
+  <si>
+    <t>Udaan Mohalla Delta Youth Club</t>
+  </si>
+  <si>
+    <t>yco2607041307m7@maildrop.cc</t>
+  </si>
+  <si>
+    <t>Jagriti Sector Nova Youth Club</t>
+  </si>
+  <si>
+    <t>yco2607041444m7@maildrop.cc</t>
   </si>
 </sst>
 </file>
@@ -1204,7 +1216,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1591,6 +1603,22 @@
         <v>63</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>67</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- now new registration for create youth club user instead of fetch from already user
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="74">
   <si>
     <t>Email</t>
   </si>
@@ -232,6 +232,24 @@
   </si>
   <si>
     <t>yco2607041444m7@maildrop.cc</t>
+  </si>
+  <si>
+    <t>Vikas Basti Elite Youth Club</t>
+  </si>
+  <si>
+    <t>ycpartnera50@maildrop.cc</t>
+  </si>
+  <si>
+    <t>Sankalp Enclave Sigma Youth Club</t>
+  </si>
+  <si>
+    <t>ycpartnera2607050024n51@maildrop.cc</t>
+  </si>
+  <si>
+    <t>Sahyog Mohalla Elite Youth Club</t>
+  </si>
+  <si>
+    <t>ycpartnera2607050051n52@maildrop.cc</t>
   </si>
 </sst>
 </file>
@@ -1216,7 +1234,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1619,6 +1637,30 @@
         <v>67</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
WIP: quiz microservice test - form fill in progress (React input issue being debugged)
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="78">
   <si>
     <t>Email</t>
   </si>
@@ -250,6 +250,18 @@
   </si>
   <si>
     <t>ycpartnera2607050051n52@maildrop.cc</t>
+  </si>
+  <si>
+    <t>Vikas Sector Delta Youth Club</t>
+  </si>
+  <si>
+    <t>ycpartnera260803203818n53@maildrop.cc</t>
+  </si>
+  <si>
+    <t>Sankalp Vihar Elite Youth Club</t>
+  </si>
+  <si>
+    <t>ycpartnera260807101411n54@maildrop.cc</t>
   </si>
 </sst>
 </file>
@@ -1234,7 +1246,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1661,6 +1673,22 @@
         <v>73</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>77</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>